<commit_message>
feat: F reporting dashboard done
</commit_message>
<xml_diff>
--- a/docs/excel_reporting/F_Reporting_Dashboard_v1.xlsx
+++ b/docs/excel_reporting/F_Reporting_Dashboard_v1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minhakim/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minhakim/Project/glucolink-a2/docs/excel_reporting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DEDADE2-76F4-5244-82FE-320AB97A2928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F21E68-DE4D-4442-A2EC-F1F05C410E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10440" yWindow="680" windowWidth="24120" windowHeight="19960" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12800" yWindow="620" windowWidth="25600" windowHeight="19280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Control" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="129">
   <si>
     <t>GlucoLink reporting export — template</t>
   </si>
@@ -97,9 +97,6 @@
     <t>UC1 rows</t>
   </si>
   <si>
-    <t>NOT RUN</t>
-  </si>
-  <si>
     <t>UC2 rows</t>
   </si>
   <si>
@@ -262,9 +259,6 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>UC2 rows 11, NON_ADHERENT 2; ADHERENT 9</t>
-  </si>
-  <si>
     <t>GL-0001</t>
   </si>
   <si>
@@ -344,6 +338,87 @@
   </si>
   <si>
     <t>Ethan Lewis</t>
+  </si>
+  <si>
+    <t>Parramatta Family Practice</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>HIGH_NO_REVIEW</t>
+  </si>
+  <si>
+    <t>HIGH_REVIEW_PENDING</t>
+  </si>
+  <si>
+    <t>Blacktown Medical Centre</t>
+  </si>
+  <si>
+    <t>OVERDUE_TEST</t>
+  </si>
+  <si>
+    <t>GL-0006</t>
+  </si>
+  <si>
+    <t>NO_TEST_ON_RECORD</t>
+  </si>
+  <si>
+    <t>GL-0014</t>
+  </si>
+  <si>
+    <t>Noah Harris</t>
+  </si>
+  <si>
+    <t>Penrith GP Clinic</t>
+  </si>
+  <si>
+    <t>RISING</t>
+  </si>
+  <si>
+    <t>STABLE</t>
+  </si>
+  <si>
+    <t>INSUFFICIENT_HISTORY</t>
+  </si>
+  <si>
+    <t>GL-0004</t>
+  </si>
+  <si>
+    <t>Olivia Brown</t>
+  </si>
+  <si>
+    <t>GL-0011</t>
+  </si>
+  <si>
+    <t>Emily Davis</t>
+  </si>
+  <si>
+    <t>GL-0013</t>
+  </si>
+  <si>
+    <t>Chloe White</t>
+  </si>
+  <si>
+    <t>GL-0015</t>
+  </si>
+  <si>
+    <t>Ava Robinson</t>
+  </si>
+  <si>
+    <t>RESULT_NOT_RETURNED</t>
+  </si>
+  <si>
+    <t>Result OBS-0010 reported 2026-06-03 has no delivery record to a clinic</t>
+  </si>
+  <si>
+    <t>MULTI_PHARMACY_OVERLAP</t>
+  </si>
+  <si>
+    <t>biguanide supplied by pharmacies 1 and 2 with overlapping supply from 2026-04-20</t>
+  </si>
+  <si>
+    <t>4/20/26</t>
   </si>
 </sst>
 </file>
@@ -353,7 +428,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -371,6 +446,11 @@
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="3">
@@ -413,7 +493,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -423,6 +503,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -859,131 +941,151 @@
       <c r="B4" s="2">
         <v>8</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="2">
+        <v>8</v>
+      </c>
       <c r="D4" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>76</v>
+        <v>21</v>
+      </c>
+      <c r="B5" s="2">
+        <v>11</v>
       </c>
       <c r="C5" s="2">
         <v>11</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" s="2">
         <v>16</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="2">
+        <v>16</v>
+      </c>
       <c r="D6" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="2">
         <v>2</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="2">
+        <v>2</v>
+      </c>
       <c r="D7" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="D8" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="D9" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="D10" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="2">
         <v>2</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="2">
+        <v>2</v>
+      </c>
       <c r="D11" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="D12" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="D13" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="D14" s="2" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1002,42 +1104,42 @@
   <sheetData>
     <row r="1" spans="1:2" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1047,7 +1149,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="8" width="28" customWidth="1"/>
@@ -1055,28 +1157,236 @@
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>55</v>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="4">
+        <v>46162</v>
+      </c>
+      <c r="E2" s="3">
+        <v>62</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H2" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" s="4">
+        <v>46204</v>
+      </c>
+      <c r="E3" s="3">
+        <v>58</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H3" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="4">
+        <v>45992</v>
+      </c>
+      <c r="E4" s="3">
+        <v>51</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="H4" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" s="4">
+        <v>46054</v>
+      </c>
+      <c r="E6" s="3">
+        <v>52</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="H6" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="4">
+        <v>46152</v>
+      </c>
+      <c r="E7" s="3">
+        <v>57</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H7" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D8" s="4">
+        <v>46244</v>
+      </c>
+      <c r="E8" s="3">
+        <v>58</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H8" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="4">
+        <v>46178</v>
+      </c>
+      <c r="E9" s="3">
+        <v>65</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H9" s="4">
+        <v>46266</v>
       </c>
     </row>
   </sheetData>
@@ -1095,48 +1405,48 @@
   <sheetData>
     <row r="1" spans="1:11" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="D2" s="3">
         <v>7</v>
@@ -1151,7 +1461,7 @@
         <v>0.98899999999999999</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I2" s="4">
         <v>46086</v>
@@ -1165,13 +1475,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D3" s="3">
         <v>3</v>
@@ -1186,7 +1496,7 @@
         <v>0.33300000000000002</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I3" s="4">
         <v>46086</v>
@@ -1200,13 +1510,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D4" s="3">
         <v>6</v>
@@ -1221,7 +1531,7 @@
         <v>0.97799999999999998</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I4" s="4">
         <v>46086</v>
@@ -1235,13 +1545,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D5" s="3">
         <v>8</v>
@@ -1256,7 +1566,7 @@
         <v>0.97199999999999998</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I5" s="4">
         <v>46086</v>
@@ -1270,13 +1580,13 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>88</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="D6" s="3">
         <v>6</v>
@@ -1291,7 +1601,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I6" s="4">
         <v>46086</v>
@@ -1305,13 +1615,13 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D7" s="3">
         <v>6</v>
@@ -1326,7 +1636,7 @@
         <v>0.97799999999999998</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I7" s="4">
         <v>46086</v>
@@ -1340,13 +1650,13 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D8" s="3">
         <v>7</v>
@@ -1361,7 +1671,7 @@
         <v>1</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I8" s="4">
         <v>46086</v>
@@ -1375,13 +1685,13 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D9" s="3">
         <v>3</v>
@@ -1396,7 +1706,7 @@
         <v>0.5</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I9" s="4">
         <v>46086</v>
@@ -1410,13 +1720,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D10" s="3">
         <v>6</v>
@@ -1431,7 +1741,7 @@
         <v>0.97199999999999998</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I10" s="4">
         <v>46086</v>
@@ -1445,13 +1755,13 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>101</v>
       </c>
       <c r="D11" s="3">
         <v>7</v>
@@ -1466,7 +1776,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I11" s="4">
         <v>46086</v>
@@ -1480,13 +1790,13 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D12" s="3">
         <v>6</v>
@@ -1501,7 +1811,7 @@
         <v>0.91700000000000004</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="I12" s="4">
         <v>46086</v>
@@ -1521,7 +1831,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="12" width="28" customWidth="1"/>
@@ -1529,40 +1839,648 @@
   <sheetData>
     <row r="1" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="3">
+        <v>3</v>
+      </c>
+      <c r="D2" s="4">
+        <v>45940</v>
+      </c>
+      <c r="E2" s="3">
+        <v>50</v>
+      </c>
+      <c r="F2" s="4">
+        <v>46162</v>
+      </c>
+      <c r="G2" s="3">
+        <v>62</v>
+      </c>
+      <c r="H2" s="3">
+        <v>12</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="3">
+        <v>0.98899999999999999</v>
+      </c>
+      <c r="K2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" s="3">
+        <v>3</v>
+      </c>
+      <c r="D3" s="4">
+        <v>45981</v>
+      </c>
+      <c r="E3" s="3">
+        <v>58</v>
+      </c>
+      <c r="F3" s="4">
+        <v>46204</v>
+      </c>
+      <c r="G3" s="3">
+        <v>58</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J3" s="3">
+        <v>0.33300000000000002</v>
+      </c>
+      <c r="K3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4">
+        <v>45992</v>
+      </c>
+      <c r="E4" s="3">
+        <v>51</v>
+      </c>
+      <c r="F4" s="4">
+        <v>45992</v>
+      </c>
+      <c r="G4" s="3">
+        <v>51</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J4" s="3">
+        <v>0.97799999999999998</v>
+      </c>
+      <c r="K4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
+        <v>45993</v>
+      </c>
+      <c r="E5" s="3">
+        <v>47</v>
+      </c>
+      <c r="F5" s="4">
+        <v>46175</v>
+      </c>
+      <c r="G5" s="3">
+        <v>48</v>
+      </c>
+      <c r="H5" s="3">
+        <v>1</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="K5" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2</v>
+      </c>
+      <c r="D6" s="4">
+        <v>46027</v>
+      </c>
+      <c r="E6" s="3">
+        <v>50.8</v>
+      </c>
+      <c r="F6" s="4">
+        <v>46147</v>
+      </c>
+      <c r="G6" s="3">
+        <v>51.9</v>
+      </c>
+      <c r="H6" s="3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J6" s="3">
+        <v>0.97199999999999998</v>
+      </c>
+      <c r="K6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="3">
+        <v>1</v>
+      </c>
+      <c r="D7" s="4">
+        <v>46157</v>
+      </c>
+      <c r="E7" s="3">
+        <v>47.5</v>
+      </c>
+      <c r="F7" s="4">
+        <v>46157</v>
+      </c>
+      <c r="G7" s="3">
+        <v>47.5</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J7" s="3">
+        <v>1</v>
+      </c>
+      <c r="K7" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2</v>
+      </c>
+      <c r="D8" s="4">
+        <v>46042</v>
+      </c>
+      <c r="E8" s="3">
+        <v>51</v>
+      </c>
+      <c r="F8" s="4">
+        <v>46198</v>
+      </c>
+      <c r="G8" s="3">
+        <v>50</v>
+      </c>
+      <c r="H8" s="3">
+        <v>-1</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J8" s="3">
+        <v>0.97799999999999998</v>
+      </c>
+      <c r="K8" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="3">
+        <v>4</v>
+      </c>
+      <c r="D9" s="4">
+        <v>45928</v>
+      </c>
+      <c r="E9" s="3">
         <v>49</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="F9" s="4">
+        <v>46201</v>
+      </c>
+      <c r="G9" s="3">
+        <v>48</v>
+      </c>
+      <c r="H9" s="3">
+        <v>-1</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J9" s="3">
+        <v>1</v>
+      </c>
+      <c r="K9" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="3">
+        <v>1</v>
+      </c>
+      <c r="D10" s="4">
+        <v>46054</v>
+      </c>
+      <c r="E10" s="3">
+        <v>52</v>
+      </c>
+      <c r="F10" s="4">
+        <v>46054</v>
+      </c>
+      <c r="G10" s="3">
+        <v>52</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J10" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K10" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="3">
+        <v>2</v>
+      </c>
+      <c r="D11" s="4">
+        <v>46096</v>
+      </c>
+      <c r="E11" s="3">
+        <v>54</v>
+      </c>
+      <c r="F11" s="4">
+        <v>46193</v>
+      </c>
+      <c r="G11" s="3">
+        <v>50</v>
+      </c>
+      <c r="H11" s="3">
+        <v>-4</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="K11" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L11" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" s="3">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4">
+        <v>46152</v>
+      </c>
+      <c r="E12" s="3">
+        <v>57</v>
+      </c>
+      <c r="F12" s="4">
+        <v>46152</v>
+      </c>
+      <c r="G12" s="3">
+        <v>57</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0.97199999999999998</v>
+      </c>
+      <c r="K12" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" s="3">
+        <v>2</v>
+      </c>
+      <c r="D13" s="4">
+        <v>45971</v>
+      </c>
+      <c r="E13" s="3">
+        <v>55</v>
+      </c>
+      <c r="F13" s="4">
+        <v>46122</v>
+      </c>
+      <c r="G13" s="3">
+        <v>60</v>
+      </c>
+      <c r="H13" s="3">
+        <v>5</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="K13" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="3">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4">
+        <v>46063</v>
+      </c>
+      <c r="E14" s="3">
+        <v>52</v>
+      </c>
+      <c r="F14" s="4">
+        <v>46244</v>
+      </c>
+      <c r="G14" s="3">
+        <v>58</v>
+      </c>
+      <c r="H14" s="3">
+        <v>6</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="K14" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L14" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="3">
+        <v>2</v>
+      </c>
+      <c r="D15" s="4">
+        <v>46113</v>
+      </c>
+      <c r="E15" s="3">
+        <v>51</v>
+      </c>
+      <c r="F15" s="4">
+        <v>46204</v>
+      </c>
+      <c r="G15" s="3">
+        <v>50</v>
+      </c>
+      <c r="H15" s="3">
+        <v>-1</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="K15" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C16" s="3">
+        <v>2</v>
+      </c>
+      <c r="D16" s="4">
+        <v>45966</v>
+      </c>
+      <c r="E16" s="3">
+        <v>53</v>
+      </c>
+      <c r="F16" s="4">
+        <v>46178</v>
+      </c>
+      <c r="G16" s="3">
         <v>65</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>55</v>
+      <c r="H16" s="3">
+        <v>12</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="J16" s="3">
+        <v>1</v>
+      </c>
+      <c r="K16" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" s="4">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C17" s="3">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4">
+        <v>46137</v>
+      </c>
+      <c r="E17" s="3">
+        <v>49</v>
+      </c>
+      <c r="F17" s="4">
+        <v>46137</v>
+      </c>
+      <c r="G17" s="3">
+        <v>49</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J17" s="3">
+        <v>0.91700000000000004</v>
+      </c>
+      <c r="K17" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" s="4">
+        <v>46266</v>
       </c>
     </row>
   </sheetData>
@@ -1573,7 +2491,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="28" customWidth="1"/>
@@ -1581,19 +2499,53 @@
   <sheetData>
     <row r="1" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>74</v>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" s="6">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix minor typo errors
</commit_message>
<xml_diff>
--- a/docs/excel_reporting/F_Reporting_Dashboard_v1.xlsx
+++ b/docs/excel_reporting/F_Reporting_Dashboard_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minhakim/Project/glucolink-a2/docs/excel_reporting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44BAC49-4570-CC41-83F3-D51EA4CB1AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67D4A2A-AD1B-954C-9924-A391F14B91A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="20160" windowHeight="19280" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19360" yWindow="740" windowWidth="20160" windowHeight="19280" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Control" sheetId="1" r:id="rId1"/>
@@ -30,14 +30,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'UC2'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'UC3'!$A$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UC4'!$A$1:$E$1</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">'UC1 Dashboard'!$A$6:$A$9</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'UC1 Dashboard'!$B$5</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'UC1 Dashboard'!$B$6:$B$9</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'UC1 Dashboard'!$A$6:$A$9</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'UC1 Dashboard'!$B$5</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'UC1 Dashboard'!$B$6:$B$9</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -55,7 +49,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -77,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="165">
   <si>
     <t>Status</t>
   </si>
@@ -566,6 +560,12 @@
   </si>
   <si>
     <t>breaks</t>
+  </si>
+  <si>
+    <t>Source: reporting.vw_uc3_hba1c_trend | database: glucolink_a2 | commit: 9a499ce | exported 2026-10-14 17:12 | checks: ALL PASS</t>
+  </si>
+  <si>
+    <t>Source: reporting.vw_care_path_breaks | database: glucolink_a2 | commit: 9a499ce | exported 2026-10-14 17:12 | checks: ALL PASS</t>
   </si>
 </sst>
 </file>
@@ -574,8 +574,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
-    <numFmt numFmtId="171" formatCode="d/mm/yyyy;@"/>
-    <numFmt numFmtId="173" formatCode="\+0.00;\-0.00;0"/>
+    <numFmt numFmtId="165" formatCode="d/mm/yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="\+0.00;\-0.00;0"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -848,7 +848,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -885,40 +885,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -926,19 +925,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1467,7 +1461,7 @@
             </a:r>
             <a:r>
               <a:rPr lang="en-US" altLang="ko-KR" baseline="0"/>
-              <a:t>per. atient,</a:t>
+              <a:t>per patient,</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="ko-KR" altLang="en-US" baseline="0"/>
@@ -1514,7 +1508,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-AU" altLang="ko-KR"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2059,7 +2053,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-AU"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2622,7 +2616,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -6385,7 +6379,7 @@
         <v>123</v>
       </c>
       <c r="E2" s="6">
-        <v>46087</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -6680,43 +6674,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="39" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="15"/>
@@ -6781,7 +6775,7 @@
       <c r="C26" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="D26" s="24" t="s">
+      <c r="D26" s="22" t="s">
         <v>48</v>
       </c>
       <c r="E26" s="14" t="s">
@@ -6807,7 +6801,7 @@
         <f>IF('UC1'!C2="","",'UC1'!C2)</f>
         <v>Parramatta Family Practice</v>
       </c>
-      <c r="D27" s="25">
+      <c r="D27" s="23">
         <f>IF('UC1'!D2="","",'UC1'!D2)</f>
         <v>46162</v>
       </c>
@@ -6837,7 +6831,7 @@
         <f>IF('UC1'!C3="","",'UC1'!C3)</f>
         <v>Parramatta Family Practice</v>
       </c>
-      <c r="D28" s="25">
+      <c r="D28" s="23">
         <f>IF('UC1'!D3="","",'UC1'!D3)</f>
         <v>46204</v>
       </c>
@@ -6863,7 +6857,7 @@
         <f>IF('UC1'!C4="","",'UC1'!C4)</f>
         <v>Blacktown Medical Centre</v>
       </c>
-      <c r="D29" s="25">
+      <c r="D29" s="23">
         <f>IF('UC1'!D4="","",'UC1'!D4)</f>
         <v>45992</v>
       </c>
@@ -6889,7 +6883,7 @@
         <f>IF('UC1'!C5="","",'UC1'!C5)</f>
         <v>Parramatta Family Practice</v>
       </c>
-      <c r="D30" s="25" t="str">
+      <c r="D30" s="23" t="str">
         <f>IF('UC1'!D5="","",'UC1'!D5)</f>
         <v/>
       </c>
@@ -6915,7 +6909,7 @@
         <f>IF('UC1'!C6="","",'UC1'!C6)</f>
         <v>Blacktown Medical Centre</v>
       </c>
-      <c r="D31" s="25">
+      <c r="D31" s="23">
         <f>IF('UC1'!D6="","",'UC1'!D6)</f>
         <v>46054</v>
       </c>
@@ -6941,7 +6935,7 @@
         <f>IF('UC1'!C7="","",'UC1'!C7)</f>
         <v>Parramatta Family Practice</v>
       </c>
-      <c r="D32" s="25">
+      <c r="D32" s="23">
         <f>IF('UC1'!D7="","",'UC1'!D7)</f>
         <v>46152</v>
       </c>
@@ -6967,7 +6961,7 @@
         <f>IF('UC1'!C8="","",'UC1'!C8)</f>
         <v>Penrith GP Clinic</v>
       </c>
-      <c r="D33" s="25">
+      <c r="D33" s="23">
         <f>IF('UC1'!D8="","",'UC1'!D8)</f>
         <v>46244</v>
       </c>
@@ -6993,7 +6987,7 @@
         <f>IF('UC1'!C9="","",'UC1'!C9)</f>
         <v>Blacktown Medical Centre</v>
       </c>
-      <c r="D34" s="25">
+      <c r="D34" s="23">
         <f>IF('UC1'!D9="","",'UC1'!D9)</f>
         <v>46178</v>
       </c>
@@ -7033,43 +7027,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="41" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="39" t="s">
         <v>153</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
@@ -7355,591 +7349,591 @@
   <cols>
     <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="28"/>
+    <col min="5" max="5" width="10.83203125" style="24"/>
     <col min="8" max="8" width="20.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="41" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+      <c r="A2" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="45" t="s">
         <v>158</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="31" t="s">
+      <c r="G5" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="H5" s="28" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="33" t="str">
+      <c r="A6" s="29" t="str">
         <f>'UC3'!A2&amp;IF('UC3'!K2=TRUE," *","")&amp;IF('UC3'!I2="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0001 *</v>
       </c>
-      <c r="B6" s="34">
+      <c r="B6" s="24">
         <f>IF('UC3'!H2="","",'UC3'!H2)</f>
         <v>12</v>
       </c>
-      <c r="C6" s="35" t="str">
+      <c r="C6" t="str">
         <f>'UC3'!I2</f>
         <v>RISING</v>
       </c>
-      <c r="D6" s="34">
+      <c r="D6" s="24">
         <f>IF('UC3'!I2="RISING",'UC3'!H2,NA())</f>
         <v>12</v>
       </c>
-      <c r="E6" s="34" t="e">
+      <c r="E6" s="24" t="e">
         <f>IF('UC3'!I2="STABLE",'UC3'!H2,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F6" s="35">
+      <c r="F6">
         <f>'UC3'!C2</f>
         <v>3</v>
       </c>
-      <c r="G6" s="35">
+      <c r="G6">
         <f>IF('UC3'!J2="","",'UC3'!J2)</f>
         <v>0.98899999999999999</v>
       </c>
-      <c r="H6" s="36" t="b">
+      <c r="H6" s="30" t="b">
         <f>'UC3'!K2</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="33" t="str">
+      <c r="A7" s="29" t="str">
         <f>'UC3'!A3&amp;IF('UC3'!K3=TRUE," *","")&amp;IF('UC3'!I3="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0002</v>
       </c>
-      <c r="B7" s="34">
+      <c r="B7" s="24">
         <f>IF('UC3'!H3="","",'UC3'!H3)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="35" t="str">
+      <c r="C7" t="str">
         <f>'UC3'!I3</f>
         <v>STABLE</v>
       </c>
-      <c r="D7" s="34" t="e">
+      <c r="D7" s="24" t="e">
         <f>IF('UC3'!I3="RISING",'UC3'!H3,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E7" s="34">
+      <c r="E7" s="24">
         <f>IF('UC3'!I3="STABLE",'UC3'!H3,NA())</f>
         <v>0</v>
       </c>
-      <c r="F7" s="35">
+      <c r="F7">
         <f>'UC3'!C3</f>
         <v>3</v>
       </c>
-      <c r="G7" s="35">
+      <c r="G7">
         <f>IF('UC3'!J3="","",'UC3'!J3)</f>
         <v>0.33300000000000002</v>
       </c>
-      <c r="H7" s="36" t="b">
+      <c r="H7" s="30" t="b">
         <f>'UC3'!K3</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="33" t="str">
+      <c r="A8" s="29" t="str">
         <f>'UC3'!A4&amp;IF('UC3'!K4=TRUE," *","")&amp;IF('UC3'!I4="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0003 (1 test)</v>
       </c>
-      <c r="B8" s="34" t="str">
+      <c r="B8" s="24" t="str">
         <f>IF('UC3'!H4="","",'UC3'!H4)</f>
         <v/>
       </c>
-      <c r="C8" s="35" t="str">
+      <c r="C8" t="str">
         <f>'UC3'!I4</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D8" s="34" t="e">
+      <c r="D8" s="24" t="e">
         <f>IF('UC3'!I4="RISING",'UC3'!H4,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E8" s="34" t="e">
+      <c r="E8" s="24" t="e">
         <f>IF('UC3'!I4="STABLE",'UC3'!H4,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F8" s="35">
+      <c r="F8">
         <f>'UC3'!C4</f>
         <v>1</v>
       </c>
-      <c r="G8" s="35">
+      <c r="G8">
         <f>IF('UC3'!J4="","",'UC3'!J4)</f>
         <v>0.97799999999999998</v>
       </c>
-      <c r="H8" s="36" t="b">
+      <c r="H8" s="30" t="b">
         <f>'UC3'!K4</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="33" t="str">
+      <c r="A9" s="29" t="str">
         <f>'UC3'!A5&amp;IF('UC3'!K5=TRUE," *","")&amp;IF('UC3'!I5="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0004</v>
       </c>
-      <c r="B9" s="34">
+      <c r="B9" s="24">
         <f>IF('UC3'!H5="","",'UC3'!H5)</f>
         <v>1</v>
       </c>
-      <c r="C9" s="35" t="str">
+      <c r="C9" t="str">
         <f>'UC3'!I5</f>
         <v>STABLE</v>
       </c>
-      <c r="D9" s="34" t="e">
+      <c r="D9" s="24" t="e">
         <f>IF('UC3'!I5="RISING",'UC3'!H5,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E9" s="34">
+      <c r="E9" s="24">
         <f>IF('UC3'!I5="STABLE",'UC3'!H5,NA())</f>
         <v>1</v>
       </c>
-      <c r="F9" s="35">
+      <c r="F9">
         <f>'UC3'!C5</f>
         <v>2</v>
       </c>
-      <c r="G9" s="35" t="str">
+      <c r="G9" t="str">
         <f>IF('UC3'!J5="","",'UC3'!J5)</f>
         <v/>
       </c>
-      <c r="H9" s="36" t="b">
+      <c r="H9" s="30" t="b">
         <f>'UC3'!K5</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="33" t="str">
+      <c r="A10" s="29" t="str">
         <f>'UC3'!A6&amp;IF('UC3'!K6=TRUE," *","")&amp;IF('UC3'!I6="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0005</v>
       </c>
-      <c r="B10" s="34">
+      <c r="B10" s="24">
         <f>IF('UC3'!H6="","",'UC3'!H6)</f>
         <v>1.1000000000000001</v>
       </c>
-      <c r="C10" s="35" t="str">
+      <c r="C10" t="str">
         <f>'UC3'!I6</f>
         <v>STABLE</v>
       </c>
-      <c r="D10" s="34" t="e">
+      <c r="D10" s="24" t="e">
         <f>IF('UC3'!I6="RISING",'UC3'!H6,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E10" s="34">
+      <c r="E10" s="24">
         <f>IF('UC3'!I6="STABLE",'UC3'!H6,NA())</f>
         <v>1.1000000000000001</v>
       </c>
-      <c r="F10" s="35">
+      <c r="F10">
         <f>'UC3'!C6</f>
         <v>2</v>
       </c>
-      <c r="G10" s="35">
+      <c r="G10">
         <f>IF('UC3'!J6="","",'UC3'!J6)</f>
         <v>0.97199999999999998</v>
       </c>
-      <c r="H10" s="36" t="b">
+      <c r="H10" s="30" t="b">
         <f>'UC3'!K6</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="33" t="str">
+      <c r="A11" s="29" t="str">
         <f>'UC3'!A7&amp;IF('UC3'!K7=TRUE," *","")&amp;IF('UC3'!I7="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0007 (1 test)</v>
       </c>
-      <c r="B11" s="34" t="str">
+      <c r="B11" s="24" t="str">
         <f>IF('UC3'!H7="","",'UC3'!H7)</f>
         <v/>
       </c>
-      <c r="C11" s="35" t="str">
+      <c r="C11" t="str">
         <f>'UC3'!I7</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D11" s="34" t="e">
+      <c r="D11" s="24" t="e">
         <f>IF('UC3'!I7="RISING",'UC3'!H7,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E11" s="34" t="e">
+      <c r="E11" s="24" t="e">
         <f>IF('UC3'!I7="STABLE",'UC3'!H7,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F11" s="35">
+      <c r="F11">
         <f>'UC3'!C7</f>
         <v>1</v>
       </c>
-      <c r="G11" s="35">
+      <c r="G11">
         <f>IF('UC3'!J7="","",'UC3'!J7)</f>
         <v>1</v>
       </c>
-      <c r="H11" s="36" t="b">
+      <c r="H11" s="30" t="b">
         <f>'UC3'!K7</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="33" t="str">
+      <c r="A12" s="29" t="str">
         <f>'UC3'!A8&amp;IF('UC3'!K8=TRUE," *","")&amp;IF('UC3'!I8="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0008</v>
       </c>
-      <c r="B12" s="34">
+      <c r="B12" s="24">
         <f>IF('UC3'!H8="","",'UC3'!H8)</f>
         <v>-1</v>
       </c>
-      <c r="C12" s="35" t="str">
+      <c r="C12" t="str">
         <f>'UC3'!I8</f>
         <v>STABLE</v>
       </c>
-      <c r="D12" s="34" t="e">
+      <c r="D12" s="24" t="e">
         <f>IF('UC3'!I8="RISING",'UC3'!H8,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E12" s="34">
+      <c r="E12" s="24">
         <f>IF('UC3'!I8="STABLE",'UC3'!H8,NA())</f>
         <v>-1</v>
       </c>
-      <c r="F12" s="35">
+      <c r="F12">
         <f>'UC3'!C8</f>
         <v>2</v>
       </c>
-      <c r="G12" s="35">
+      <c r="G12">
         <f>IF('UC3'!J8="","",'UC3'!J8)</f>
         <v>0.97799999999999998</v>
       </c>
-      <c r="H12" s="36" t="b">
+      <c r="H12" s="30" t="b">
         <f>'UC3'!K8</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="33" t="str">
+      <c r="A13" s="29" t="str">
         <f>'UC3'!A9&amp;IF('UC3'!K9=TRUE," *","")&amp;IF('UC3'!I9="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0009</v>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="24">
         <f>IF('UC3'!H9="","",'UC3'!H9)</f>
         <v>-1</v>
       </c>
-      <c r="C13" s="35" t="str">
+      <c r="C13" t="str">
         <f>'UC3'!I9</f>
         <v>STABLE</v>
       </c>
-      <c r="D13" s="34" t="e">
+      <c r="D13" s="24" t="e">
         <f>IF('UC3'!I9="RISING",'UC3'!H9,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E13" s="34">
+      <c r="E13" s="24">
         <f>IF('UC3'!I9="STABLE",'UC3'!H9,NA())</f>
         <v>-1</v>
       </c>
-      <c r="F13" s="35">
+      <c r="F13">
         <f>'UC3'!C9</f>
         <v>4</v>
       </c>
-      <c r="G13" s="35">
+      <c r="G13">
         <f>IF('UC3'!J9="","",'UC3'!J9)</f>
         <v>1</v>
       </c>
-      <c r="H13" s="36" t="b">
+      <c r="H13" s="30" t="b">
         <f>'UC3'!K9</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="33" t="str">
+      <c r="A14" s="29" t="str">
         <f>'UC3'!A10&amp;IF('UC3'!K10=TRUE," *","")&amp;IF('UC3'!I10="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0010 (1 test)</v>
       </c>
-      <c r="B14" s="34" t="str">
+      <c r="B14" s="24" t="str">
         <f>IF('UC3'!H10="","",'UC3'!H10)</f>
         <v/>
       </c>
-      <c r="C14" s="35" t="str">
+      <c r="C14" t="str">
         <f>'UC3'!I10</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D14" s="34" t="e">
+      <c r="D14" s="24" t="e">
         <f>IF('UC3'!I10="RISING",'UC3'!H10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E14" s="34" t="e">
+      <c r="E14" s="24" t="e">
         <f>IF('UC3'!I10="STABLE",'UC3'!H10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F14" s="35">
+      <c r="F14">
         <f>'UC3'!C10</f>
         <v>1</v>
       </c>
-      <c r="G14" s="35">
+      <c r="G14">
         <f>IF('UC3'!J10="","",'UC3'!J10)</f>
         <v>0.5</v>
       </c>
-      <c r="H14" s="36" t="b">
+      <c r="H14" s="30" t="b">
         <f>'UC3'!K10</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="33" t="str">
+      <c r="A15" s="29" t="str">
         <f>'UC3'!A11&amp;IF('UC3'!K11=TRUE," *","")&amp;IF('UC3'!I11="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0011</v>
       </c>
-      <c r="B15" s="34">
+      <c r="B15" s="24">
         <f>IF('UC3'!H11="","",'UC3'!H11)</f>
         <v>-4</v>
       </c>
-      <c r="C15" s="35" t="str">
+      <c r="C15" t="str">
         <f>'UC3'!I11</f>
         <v>STABLE</v>
       </c>
-      <c r="D15" s="34" t="e">
+      <c r="D15" s="24" t="e">
         <f>IF('UC3'!I11="RISING",'UC3'!H11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E15" s="34">
+      <c r="E15" s="24">
         <f>IF('UC3'!I11="STABLE",'UC3'!H11,NA())</f>
         <v>-4</v>
       </c>
-      <c r="F15" s="35">
+      <c r="F15">
         <f>'UC3'!C11</f>
         <v>2</v>
       </c>
-      <c r="G15" s="35" t="str">
+      <c r="G15" t="str">
         <f>IF('UC3'!J11="","",'UC3'!J11)</f>
         <v/>
       </c>
-      <c r="H15" s="36" t="b">
+      <c r="H15" s="30" t="b">
         <f>'UC3'!K11</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="33" t="str">
+      <c r="A16" s="29" t="str">
         <f>'UC3'!A12&amp;IF('UC3'!K12=TRUE," *","")&amp;IF('UC3'!I12="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0012 (1 test)</v>
       </c>
-      <c r="B16" s="34" t="str">
+      <c r="B16" s="24" t="str">
         <f>IF('UC3'!H12="","",'UC3'!H12)</f>
         <v/>
       </c>
-      <c r="C16" s="35" t="str">
+      <c r="C16" t="str">
         <f>'UC3'!I12</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D16" s="34" t="e">
+      <c r="D16" s="24" t="e">
         <f>IF('UC3'!I12="RISING",'UC3'!H12,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E16" s="34" t="e">
+      <c r="E16" s="24" t="e">
         <f>IF('UC3'!I12="STABLE",'UC3'!H12,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F16" s="35">
+      <c r="F16">
         <f>'UC3'!C12</f>
         <v>1</v>
       </c>
-      <c r="G16" s="35">
+      <c r="G16">
         <f>IF('UC3'!J12="","",'UC3'!J12)</f>
         <v>0.97199999999999998</v>
       </c>
-      <c r="H16" s="36" t="b">
+      <c r="H16" s="30" t="b">
         <f>'UC3'!K12</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="33" t="str">
+      <c r="A17" s="29" t="str">
         <f>'UC3'!A13&amp;IF('UC3'!K13=TRUE," *","")&amp;IF('UC3'!I13="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0013</v>
       </c>
-      <c r="B17" s="34">
+      <c r="B17" s="24">
         <f>IF('UC3'!H13="","",'UC3'!H13)</f>
         <v>5</v>
       </c>
-      <c r="C17" s="35" t="str">
+      <c r="C17" t="str">
         <f>'UC3'!I13</f>
         <v>RISING</v>
       </c>
-      <c r="D17" s="34">
+      <c r="D17" s="24">
         <f>IF('UC3'!I13="RISING",'UC3'!H13,NA())</f>
         <v>5</v>
       </c>
-      <c r="E17" s="34" t="e">
+      <c r="E17" s="24" t="e">
         <f>IF('UC3'!I13="STABLE",'UC3'!H13,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F17" s="35">
+      <c r="F17">
         <f>'UC3'!C13</f>
         <v>2</v>
       </c>
-      <c r="G17" s="35" t="str">
+      <c r="G17" t="str">
         <f>IF('UC3'!J13="","",'UC3'!J13)</f>
         <v/>
       </c>
-      <c r="H17" s="36" t="b">
+      <c r="H17" s="30" t="b">
         <f>'UC3'!K13</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="33" t="str">
+      <c r="A18" s="29" t="str">
         <f>'UC3'!A14&amp;IF('UC3'!K14=TRUE," *","")&amp;IF('UC3'!I14="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0014</v>
       </c>
-      <c r="B18" s="34">
+      <c r="B18" s="24">
         <f>IF('UC3'!H14="","",'UC3'!H14)</f>
         <v>6</v>
       </c>
-      <c r="C18" s="35" t="str">
+      <c r="C18" t="str">
         <f>'UC3'!I14</f>
         <v>RISING</v>
       </c>
-      <c r="D18" s="34">
+      <c r="D18" s="24">
         <f>IF('UC3'!I14="RISING",'UC3'!H14,NA())</f>
         <v>6</v>
       </c>
-      <c r="E18" s="34" t="e">
+      <c r="E18" s="24" t="e">
         <f>IF('UC3'!I14="STABLE",'UC3'!H14,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F18" s="35">
+      <c r="F18">
         <f>'UC3'!C14</f>
         <v>2</v>
       </c>
-      <c r="G18" s="35" t="str">
+      <c r="G18" t="str">
         <f>IF('UC3'!J14="","",'UC3'!J14)</f>
         <v/>
       </c>
-      <c r="H18" s="36" t="b">
+      <c r="H18" s="30" t="b">
         <f>'UC3'!K14</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="33" t="str">
+      <c r="A19" s="29" t="str">
         <f>'UC3'!A15&amp;IF('UC3'!K15=TRUE," *","")&amp;IF('UC3'!I15="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0015</v>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="24">
         <f>IF('UC3'!H15="","",'UC3'!H15)</f>
         <v>-1</v>
       </c>
-      <c r="C19" s="35" t="str">
+      <c r="C19" t="str">
         <f>'UC3'!I15</f>
         <v>STABLE</v>
       </c>
-      <c r="D19" s="34" t="e">
+      <c r="D19" s="24" t="e">
         <f>IF('UC3'!I15="RISING",'UC3'!H15,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E19" s="34">
+      <c r="E19" s="24">
         <f>IF('UC3'!I15="STABLE",'UC3'!H15,NA())</f>
         <v>-1</v>
       </c>
-      <c r="F19" s="35">
+      <c r="F19">
         <f>'UC3'!C15</f>
         <v>2</v>
       </c>
-      <c r="G19" s="35" t="str">
+      <c r="G19" t="str">
         <f>IF('UC3'!J15="","",'UC3'!J15)</f>
         <v/>
       </c>
-      <c r="H19" s="36" t="b">
+      <c r="H19" s="30" t="b">
         <f>'UC3'!K15</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="33" t="str">
+      <c r="A20" s="29" t="str">
         <f>'UC3'!A16&amp;IF('UC3'!K16=TRUE," *","")&amp;IF('UC3'!I16="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0016 *</v>
       </c>
-      <c r="B20" s="34">
+      <c r="B20" s="24">
         <f>IF('UC3'!H16="","",'UC3'!H16)</f>
         <v>12</v>
       </c>
-      <c r="C20" s="35" t="str">
+      <c r="C20" t="str">
         <f>'UC3'!I16</f>
         <v>RISING</v>
       </c>
-      <c r="D20" s="34">
+      <c r="D20" s="24">
         <f>IF('UC3'!I16="RISING",'UC3'!H16,NA())</f>
         <v>12</v>
       </c>
-      <c r="E20" s="34" t="e">
+      <c r="E20" s="24" t="e">
         <f>IF('UC3'!I16="STABLE",'UC3'!H16,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F20" s="35">
+      <c r="F20">
         <f>'UC3'!C16</f>
         <v>2</v>
       </c>
-      <c r="G20" s="35">
+      <c r="G20">
         <f>IF('UC3'!J16="","",'UC3'!J16)</f>
         <v>1</v>
       </c>
-      <c r="H20" s="36" t="b">
+      <c r="H20" s="30" t="b">
         <f>'UC3'!K16</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="37" t="str">
+      <c r="A21" s="31" t="str">
         <f>'UC3'!A17&amp;IF('UC3'!K17=TRUE," *","")&amp;IF('UC3'!I17="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0017 (1 test)</v>
       </c>
-      <c r="B21" s="38" t="str">
+      <c r="B21" s="32" t="str">
         <f>IF('UC3'!H17="","",'UC3'!H17)</f>
         <v/>
       </c>
@@ -7947,11 +7941,11 @@
         <f>'UC3'!I17</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D21" s="38" t="e">
+      <c r="D21" s="32" t="e">
         <f>IF('UC3'!I17="RISING",'UC3'!H17,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E21" s="38" t="e">
+      <c r="E21" s="32" t="e">
         <f>IF('UC3'!I17="STABLE",'UC3'!H17,NA())</f>
         <v>#N/A</v>
       </c>
@@ -7963,22 +7957,22 @@
         <f>IF('UC3'!J17="","",'UC3'!J17)</f>
         <v>0.91700000000000004</v>
       </c>
-      <c r="H21" s="39" t="b">
+      <c r="H21" s="33" t="b">
         <f>'UC3'!K17</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -8003,75 +7997,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="40" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
+      <c r="A2" s="39" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="35"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="28" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="B6" s="36">
+      <c r="B6" s="30">
         <f>COUNTIF('UC4'!C:C,A6)</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="39">
+      <c r="B7" s="33">
         <f>COUNTIF('UC4'!C:C,A7)</f>
         <v>1</v>
       </c>
@@ -8086,56 +8080,56 @@
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="31" t="s">
+      <c r="C24" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="D24" s="31" t="s">
+      <c r="D24" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="E24" s="43" t="s">
+      <c r="E24" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="43"/>
-      <c r="I24" s="43"/>
-      <c r="J24" s="44"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="43"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="33" t="str">
+      <c r="A25" s="29" t="str">
         <f>IF('UC4'!A2="","",'UC4'!A2)</f>
         <v>GL-0004</v>
       </c>
-      <c r="B25" s="35" t="str">
+      <c r="B25" t="str">
         <f>IF('UC4'!B2="","",'UC4'!B2)</f>
         <v>Olivia Brown</v>
       </c>
-      <c r="C25" s="35" t="str">
+      <c r="C25" t="str">
         <f>IF('UC4'!C2="","",'UC4'!C2)</f>
         <v>RESULT_NOT_RETURNED</v>
       </c>
-      <c r="D25" s="45">
+      <c r="D25" s="8">
         <f>IF('UC4'!E2="","",'UC4'!E2)</f>
-        <v>46087</v>
-      </c>
-      <c r="E25" s="46" t="str">
+        <v>46176</v>
+      </c>
+      <c r="E25" s="35" t="str">
         <f>IF('UC4'!D2="","",'UC4'!D2)</f>
         <v>Result OBS-0010 reported 2026-06-03 has no delivery record to a clinic</v>
       </c>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="47"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="35"/>
+      <c r="H25" s="35"/>
+      <c r="I25" s="35"/>
+      <c r="J25" s="36"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="37" t="str">
+      <c r="A26" s="31" t="str">
         <f>IF('UC4'!A3="","",'UC4'!A3)</f>
         <v>GL-0005</v>
       </c>
@@ -8147,19 +8141,19 @@
         <f>IF('UC4'!C3="","",'UC4'!C3)</f>
         <v>MULTI_PHARMACY_OVERLAP</v>
       </c>
-      <c r="D26" s="48">
+      <c r="D26" s="34">
         <f>IF('UC4'!E3="","",'UC4'!E3)</f>
         <v>46132</v>
       </c>
-      <c r="E26" s="49" t="str">
+      <c r="E26" s="37" t="str">
         <f>IF('UC4'!D3="","",'UC4'!D3)</f>
         <v>biguanide supplied by pharmacies 1 and 2 with overlapping supply from 2026-04-20</v>
       </c>
-      <c r="F26" s="49"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="49"/>
-      <c r="I26" s="49"/>
-      <c r="J26" s="50"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="37"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
fix minor typo errors (#16)
</commit_message>
<xml_diff>
--- a/docs/excel_reporting/F_Reporting_Dashboard_v1.xlsx
+++ b/docs/excel_reporting/F_Reporting_Dashboard_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minhakim/Project/glucolink-a2/docs/excel_reporting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44BAC49-4570-CC41-83F3-D51EA4CB1AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67D4A2A-AD1B-954C-9924-A391F14B91A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="20160" windowHeight="19280" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19360" yWindow="740" windowWidth="20160" windowHeight="19280" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Control" sheetId="1" r:id="rId1"/>
@@ -30,14 +30,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'UC2'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'UC3'!$A$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UC4'!$A$1:$E$1</definedName>
-    <definedName name="_xlchart.v1.0" hidden="1">'UC1 Dashboard'!$A$6:$A$9</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'UC1 Dashboard'!$B$5</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'UC1 Dashboard'!$B$6:$B$9</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'UC1 Dashboard'!$A$6:$A$9</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'UC1 Dashboard'!$B$5</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'UC1 Dashboard'!$B$6:$B$9</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -55,7 +49,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -77,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="165">
   <si>
     <t>Status</t>
   </si>
@@ -566,6 +560,12 @@
   </si>
   <si>
     <t>breaks</t>
+  </si>
+  <si>
+    <t>Source: reporting.vw_uc3_hba1c_trend | database: glucolink_a2 | commit: 9a499ce | exported 2026-10-14 17:12 | checks: ALL PASS</t>
+  </si>
+  <si>
+    <t>Source: reporting.vw_care_path_breaks | database: glucolink_a2 | commit: 9a499ce | exported 2026-10-14 17:12 | checks: ALL PASS</t>
   </si>
 </sst>
 </file>
@@ -574,8 +574,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
-    <numFmt numFmtId="171" formatCode="d/mm/yyyy;@"/>
-    <numFmt numFmtId="173" formatCode="\+0.00;\-0.00;0"/>
+    <numFmt numFmtId="165" formatCode="d/mm/yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="\+0.00;\-0.00;0"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -848,7 +848,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -885,40 +885,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -926,19 +925,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1467,7 +1461,7 @@
             </a:r>
             <a:r>
               <a:rPr lang="en-US" altLang="ko-KR" baseline="0"/>
-              <a:t>per. atient,</a:t>
+              <a:t>per patient,</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="ko-KR" altLang="en-US" baseline="0"/>
@@ -1514,7 +1508,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-AU" altLang="ko-KR"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2059,7 +2053,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-AU"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2622,7 +2616,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -6385,7 +6379,7 @@
         <v>123</v>
       </c>
       <c r="E2" s="6">
-        <v>46087</v>
+        <v>46176</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -6680,43 +6674,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="44" t="s">
         <v>147</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="39" t="s">
         <v>148</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="39" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="15"/>
@@ -6781,7 +6775,7 @@
       <c r="C26" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="D26" s="24" t="s">
+      <c r="D26" s="22" t="s">
         <v>48</v>
       </c>
       <c r="E26" s="14" t="s">
@@ -6807,7 +6801,7 @@
         <f>IF('UC1'!C2="","",'UC1'!C2)</f>
         <v>Parramatta Family Practice</v>
       </c>
-      <c r="D27" s="25">
+      <c r="D27" s="23">
         <f>IF('UC1'!D2="","",'UC1'!D2)</f>
         <v>46162</v>
       </c>
@@ -6837,7 +6831,7 @@
         <f>IF('UC1'!C3="","",'UC1'!C3)</f>
         <v>Parramatta Family Practice</v>
       </c>
-      <c r="D28" s="25">
+      <c r="D28" s="23">
         <f>IF('UC1'!D3="","",'UC1'!D3)</f>
         <v>46204</v>
       </c>
@@ -6863,7 +6857,7 @@
         <f>IF('UC1'!C4="","",'UC1'!C4)</f>
         <v>Blacktown Medical Centre</v>
       </c>
-      <c r="D29" s="25">
+      <c r="D29" s="23">
         <f>IF('UC1'!D4="","",'UC1'!D4)</f>
         <v>45992</v>
       </c>
@@ -6889,7 +6883,7 @@
         <f>IF('UC1'!C5="","",'UC1'!C5)</f>
         <v>Parramatta Family Practice</v>
       </c>
-      <c r="D30" s="25" t="str">
+      <c r="D30" s="23" t="str">
         <f>IF('UC1'!D5="","",'UC1'!D5)</f>
         <v/>
       </c>
@@ -6915,7 +6909,7 @@
         <f>IF('UC1'!C6="","",'UC1'!C6)</f>
         <v>Blacktown Medical Centre</v>
       </c>
-      <c r="D31" s="25">
+      <c r="D31" s="23">
         <f>IF('UC1'!D6="","",'UC1'!D6)</f>
         <v>46054</v>
       </c>
@@ -6941,7 +6935,7 @@
         <f>IF('UC1'!C7="","",'UC1'!C7)</f>
         <v>Parramatta Family Practice</v>
       </c>
-      <c r="D32" s="25">
+      <c r="D32" s="23">
         <f>IF('UC1'!D7="","",'UC1'!D7)</f>
         <v>46152</v>
       </c>
@@ -6967,7 +6961,7 @@
         <f>IF('UC1'!C8="","",'UC1'!C8)</f>
         <v>Penrith GP Clinic</v>
       </c>
-      <c r="D33" s="25">
+      <c r="D33" s="23">
         <f>IF('UC1'!D8="","",'UC1'!D8)</f>
         <v>46244</v>
       </c>
@@ -6993,7 +6987,7 @@
         <f>IF('UC1'!C9="","",'UC1'!C9)</f>
         <v>Blacktown Medical Centre</v>
       </c>
-      <c r="D34" s="25">
+      <c r="D34" s="23">
         <f>IF('UC1'!D9="","",'UC1'!D9)</f>
         <v>46178</v>
       </c>
@@ -7033,43 +7027,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="41" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="39" t="s">
         <v>153</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
@@ -7355,591 +7349,591 @@
   <cols>
     <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="28"/>
+    <col min="5" max="5" width="10.83203125" style="24"/>
     <col min="8" max="8" width="20.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="41" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+      <c r="A2" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="45" t="s">
         <v>158</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="25" t="s">
         <v>155</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="31" t="s">
+      <c r="G5" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="H5" s="28" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="33" t="str">
+      <c r="A6" s="29" t="str">
         <f>'UC3'!A2&amp;IF('UC3'!K2=TRUE," *","")&amp;IF('UC3'!I2="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0001 *</v>
       </c>
-      <c r="B6" s="34">
+      <c r="B6" s="24">
         <f>IF('UC3'!H2="","",'UC3'!H2)</f>
         <v>12</v>
       </c>
-      <c r="C6" s="35" t="str">
+      <c r="C6" t="str">
         <f>'UC3'!I2</f>
         <v>RISING</v>
       </c>
-      <c r="D6" s="34">
+      <c r="D6" s="24">
         <f>IF('UC3'!I2="RISING",'UC3'!H2,NA())</f>
         <v>12</v>
       </c>
-      <c r="E6" s="34" t="e">
+      <c r="E6" s="24" t="e">
         <f>IF('UC3'!I2="STABLE",'UC3'!H2,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F6" s="35">
+      <c r="F6">
         <f>'UC3'!C2</f>
         <v>3</v>
       </c>
-      <c r="G6" s="35">
+      <c r="G6">
         <f>IF('UC3'!J2="","",'UC3'!J2)</f>
         <v>0.98899999999999999</v>
       </c>
-      <c r="H6" s="36" t="b">
+      <c r="H6" s="30" t="b">
         <f>'UC3'!K2</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="33" t="str">
+      <c r="A7" s="29" t="str">
         <f>'UC3'!A3&amp;IF('UC3'!K3=TRUE," *","")&amp;IF('UC3'!I3="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0002</v>
       </c>
-      <c r="B7" s="34">
+      <c r="B7" s="24">
         <f>IF('UC3'!H3="","",'UC3'!H3)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="35" t="str">
+      <c r="C7" t="str">
         <f>'UC3'!I3</f>
         <v>STABLE</v>
       </c>
-      <c r="D7" s="34" t="e">
+      <c r="D7" s="24" t="e">
         <f>IF('UC3'!I3="RISING",'UC3'!H3,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E7" s="34">
+      <c r="E7" s="24">
         <f>IF('UC3'!I3="STABLE",'UC3'!H3,NA())</f>
         <v>0</v>
       </c>
-      <c r="F7" s="35">
+      <c r="F7">
         <f>'UC3'!C3</f>
         <v>3</v>
       </c>
-      <c r="G7" s="35">
+      <c r="G7">
         <f>IF('UC3'!J3="","",'UC3'!J3)</f>
         <v>0.33300000000000002</v>
       </c>
-      <c r="H7" s="36" t="b">
+      <c r="H7" s="30" t="b">
         <f>'UC3'!K3</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="33" t="str">
+      <c r="A8" s="29" t="str">
         <f>'UC3'!A4&amp;IF('UC3'!K4=TRUE," *","")&amp;IF('UC3'!I4="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0003 (1 test)</v>
       </c>
-      <c r="B8" s="34" t="str">
+      <c r="B8" s="24" t="str">
         <f>IF('UC3'!H4="","",'UC3'!H4)</f>
         <v/>
       </c>
-      <c r="C8" s="35" t="str">
+      <c r="C8" t="str">
         <f>'UC3'!I4</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D8" s="34" t="e">
+      <c r="D8" s="24" t="e">
         <f>IF('UC3'!I4="RISING",'UC3'!H4,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E8" s="34" t="e">
+      <c r="E8" s="24" t="e">
         <f>IF('UC3'!I4="STABLE",'UC3'!H4,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F8" s="35">
+      <c r="F8">
         <f>'UC3'!C4</f>
         <v>1</v>
       </c>
-      <c r="G8" s="35">
+      <c r="G8">
         <f>IF('UC3'!J4="","",'UC3'!J4)</f>
         <v>0.97799999999999998</v>
       </c>
-      <c r="H8" s="36" t="b">
+      <c r="H8" s="30" t="b">
         <f>'UC3'!K4</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="33" t="str">
+      <c r="A9" s="29" t="str">
         <f>'UC3'!A5&amp;IF('UC3'!K5=TRUE," *","")&amp;IF('UC3'!I5="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0004</v>
       </c>
-      <c r="B9" s="34">
+      <c r="B9" s="24">
         <f>IF('UC3'!H5="","",'UC3'!H5)</f>
         <v>1</v>
       </c>
-      <c r="C9" s="35" t="str">
+      <c r="C9" t="str">
         <f>'UC3'!I5</f>
         <v>STABLE</v>
       </c>
-      <c r="D9" s="34" t="e">
+      <c r="D9" s="24" t="e">
         <f>IF('UC3'!I5="RISING",'UC3'!H5,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E9" s="34">
+      <c r="E9" s="24">
         <f>IF('UC3'!I5="STABLE",'UC3'!H5,NA())</f>
         <v>1</v>
       </c>
-      <c r="F9" s="35">
+      <c r="F9">
         <f>'UC3'!C5</f>
         <v>2</v>
       </c>
-      <c r="G9" s="35" t="str">
+      <c r="G9" t="str">
         <f>IF('UC3'!J5="","",'UC3'!J5)</f>
         <v/>
       </c>
-      <c r="H9" s="36" t="b">
+      <c r="H9" s="30" t="b">
         <f>'UC3'!K5</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="33" t="str">
+      <c r="A10" s="29" t="str">
         <f>'UC3'!A6&amp;IF('UC3'!K6=TRUE," *","")&amp;IF('UC3'!I6="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0005</v>
       </c>
-      <c r="B10" s="34">
+      <c r="B10" s="24">
         <f>IF('UC3'!H6="","",'UC3'!H6)</f>
         <v>1.1000000000000001</v>
       </c>
-      <c r="C10" s="35" t="str">
+      <c r="C10" t="str">
         <f>'UC3'!I6</f>
         <v>STABLE</v>
       </c>
-      <c r="D10" s="34" t="e">
+      <c r="D10" s="24" t="e">
         <f>IF('UC3'!I6="RISING",'UC3'!H6,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E10" s="34">
+      <c r="E10" s="24">
         <f>IF('UC3'!I6="STABLE",'UC3'!H6,NA())</f>
         <v>1.1000000000000001</v>
       </c>
-      <c r="F10" s="35">
+      <c r="F10">
         <f>'UC3'!C6</f>
         <v>2</v>
       </c>
-      <c r="G10" s="35">
+      <c r="G10">
         <f>IF('UC3'!J6="","",'UC3'!J6)</f>
         <v>0.97199999999999998</v>
       </c>
-      <c r="H10" s="36" t="b">
+      <c r="H10" s="30" t="b">
         <f>'UC3'!K6</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="33" t="str">
+      <c r="A11" s="29" t="str">
         <f>'UC3'!A7&amp;IF('UC3'!K7=TRUE," *","")&amp;IF('UC3'!I7="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0007 (1 test)</v>
       </c>
-      <c r="B11" s="34" t="str">
+      <c r="B11" s="24" t="str">
         <f>IF('UC3'!H7="","",'UC3'!H7)</f>
         <v/>
       </c>
-      <c r="C11" s="35" t="str">
+      <c r="C11" t="str">
         <f>'UC3'!I7</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D11" s="34" t="e">
+      <c r="D11" s="24" t="e">
         <f>IF('UC3'!I7="RISING",'UC3'!H7,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E11" s="34" t="e">
+      <c r="E11" s="24" t="e">
         <f>IF('UC3'!I7="STABLE",'UC3'!H7,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F11" s="35">
+      <c r="F11">
         <f>'UC3'!C7</f>
         <v>1</v>
       </c>
-      <c r="G11" s="35">
+      <c r="G11">
         <f>IF('UC3'!J7="","",'UC3'!J7)</f>
         <v>1</v>
       </c>
-      <c r="H11" s="36" t="b">
+      <c r="H11" s="30" t="b">
         <f>'UC3'!K7</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="33" t="str">
+      <c r="A12" s="29" t="str">
         <f>'UC3'!A8&amp;IF('UC3'!K8=TRUE," *","")&amp;IF('UC3'!I8="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0008</v>
       </c>
-      <c r="B12" s="34">
+      <c r="B12" s="24">
         <f>IF('UC3'!H8="","",'UC3'!H8)</f>
         <v>-1</v>
       </c>
-      <c r="C12" s="35" t="str">
+      <c r="C12" t="str">
         <f>'UC3'!I8</f>
         <v>STABLE</v>
       </c>
-      <c r="D12" s="34" t="e">
+      <c r="D12" s="24" t="e">
         <f>IF('UC3'!I8="RISING",'UC3'!H8,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E12" s="34">
+      <c r="E12" s="24">
         <f>IF('UC3'!I8="STABLE",'UC3'!H8,NA())</f>
         <v>-1</v>
       </c>
-      <c r="F12" s="35">
+      <c r="F12">
         <f>'UC3'!C8</f>
         <v>2</v>
       </c>
-      <c r="G12" s="35">
+      <c r="G12">
         <f>IF('UC3'!J8="","",'UC3'!J8)</f>
         <v>0.97799999999999998</v>
       </c>
-      <c r="H12" s="36" t="b">
+      <c r="H12" s="30" t="b">
         <f>'UC3'!K8</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="33" t="str">
+      <c r="A13" s="29" t="str">
         <f>'UC3'!A9&amp;IF('UC3'!K9=TRUE," *","")&amp;IF('UC3'!I9="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0009</v>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="24">
         <f>IF('UC3'!H9="","",'UC3'!H9)</f>
         <v>-1</v>
       </c>
-      <c r="C13" s="35" t="str">
+      <c r="C13" t="str">
         <f>'UC3'!I9</f>
         <v>STABLE</v>
       </c>
-      <c r="D13" s="34" t="e">
+      <c r="D13" s="24" t="e">
         <f>IF('UC3'!I9="RISING",'UC3'!H9,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E13" s="34">
+      <c r="E13" s="24">
         <f>IF('UC3'!I9="STABLE",'UC3'!H9,NA())</f>
         <v>-1</v>
       </c>
-      <c r="F13" s="35">
+      <c r="F13">
         <f>'UC3'!C9</f>
         <v>4</v>
       </c>
-      <c r="G13" s="35">
+      <c r="G13">
         <f>IF('UC3'!J9="","",'UC3'!J9)</f>
         <v>1</v>
       </c>
-      <c r="H13" s="36" t="b">
+      <c r="H13" s="30" t="b">
         <f>'UC3'!K9</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14" s="33" t="str">
+      <c r="A14" s="29" t="str">
         <f>'UC3'!A10&amp;IF('UC3'!K10=TRUE," *","")&amp;IF('UC3'!I10="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0010 (1 test)</v>
       </c>
-      <c r="B14" s="34" t="str">
+      <c r="B14" s="24" t="str">
         <f>IF('UC3'!H10="","",'UC3'!H10)</f>
         <v/>
       </c>
-      <c r="C14" s="35" t="str">
+      <c r="C14" t="str">
         <f>'UC3'!I10</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D14" s="34" t="e">
+      <c r="D14" s="24" t="e">
         <f>IF('UC3'!I10="RISING",'UC3'!H10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E14" s="34" t="e">
+      <c r="E14" s="24" t="e">
         <f>IF('UC3'!I10="STABLE",'UC3'!H10,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F14" s="35">
+      <c r="F14">
         <f>'UC3'!C10</f>
         <v>1</v>
       </c>
-      <c r="G14" s="35">
+      <c r="G14">
         <f>IF('UC3'!J10="","",'UC3'!J10)</f>
         <v>0.5</v>
       </c>
-      <c r="H14" s="36" t="b">
+      <c r="H14" s="30" t="b">
         <f>'UC3'!K10</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15" s="33" t="str">
+      <c r="A15" s="29" t="str">
         <f>'UC3'!A11&amp;IF('UC3'!K11=TRUE," *","")&amp;IF('UC3'!I11="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0011</v>
       </c>
-      <c r="B15" s="34">
+      <c r="B15" s="24">
         <f>IF('UC3'!H11="","",'UC3'!H11)</f>
         <v>-4</v>
       </c>
-      <c r="C15" s="35" t="str">
+      <c r="C15" t="str">
         <f>'UC3'!I11</f>
         <v>STABLE</v>
       </c>
-      <c r="D15" s="34" t="e">
+      <c r="D15" s="24" t="e">
         <f>IF('UC3'!I11="RISING",'UC3'!H11,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E15" s="34">
+      <c r="E15" s="24">
         <f>IF('UC3'!I11="STABLE",'UC3'!H11,NA())</f>
         <v>-4</v>
       </c>
-      <c r="F15" s="35">
+      <c r="F15">
         <f>'UC3'!C11</f>
         <v>2</v>
       </c>
-      <c r="G15" s="35" t="str">
+      <c r="G15" t="str">
         <f>IF('UC3'!J11="","",'UC3'!J11)</f>
         <v/>
       </c>
-      <c r="H15" s="36" t="b">
+      <c r="H15" s="30" t="b">
         <f>'UC3'!K11</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="33" t="str">
+      <c r="A16" s="29" t="str">
         <f>'UC3'!A12&amp;IF('UC3'!K12=TRUE," *","")&amp;IF('UC3'!I12="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0012 (1 test)</v>
       </c>
-      <c r="B16" s="34" t="str">
+      <c r="B16" s="24" t="str">
         <f>IF('UC3'!H12="","",'UC3'!H12)</f>
         <v/>
       </c>
-      <c r="C16" s="35" t="str">
+      <c r="C16" t="str">
         <f>'UC3'!I12</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D16" s="34" t="e">
+      <c r="D16" s="24" t="e">
         <f>IF('UC3'!I12="RISING",'UC3'!H12,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E16" s="34" t="e">
+      <c r="E16" s="24" t="e">
         <f>IF('UC3'!I12="STABLE",'UC3'!H12,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F16" s="35">
+      <c r="F16">
         <f>'UC3'!C12</f>
         <v>1</v>
       </c>
-      <c r="G16" s="35">
+      <c r="G16">
         <f>IF('UC3'!J12="","",'UC3'!J12)</f>
         <v>0.97199999999999998</v>
       </c>
-      <c r="H16" s="36" t="b">
+      <c r="H16" s="30" t="b">
         <f>'UC3'!K12</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="33" t="str">
+      <c r="A17" s="29" t="str">
         <f>'UC3'!A13&amp;IF('UC3'!K13=TRUE," *","")&amp;IF('UC3'!I13="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0013</v>
       </c>
-      <c r="B17" s="34">
+      <c r="B17" s="24">
         <f>IF('UC3'!H13="","",'UC3'!H13)</f>
         <v>5</v>
       </c>
-      <c r="C17" s="35" t="str">
+      <c r="C17" t="str">
         <f>'UC3'!I13</f>
         <v>RISING</v>
       </c>
-      <c r="D17" s="34">
+      <c r="D17" s="24">
         <f>IF('UC3'!I13="RISING",'UC3'!H13,NA())</f>
         <v>5</v>
       </c>
-      <c r="E17" s="34" t="e">
+      <c r="E17" s="24" t="e">
         <f>IF('UC3'!I13="STABLE",'UC3'!H13,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F17" s="35">
+      <c r="F17">
         <f>'UC3'!C13</f>
         <v>2</v>
       </c>
-      <c r="G17" s="35" t="str">
+      <c r="G17" t="str">
         <f>IF('UC3'!J13="","",'UC3'!J13)</f>
         <v/>
       </c>
-      <c r="H17" s="36" t="b">
+      <c r="H17" s="30" t="b">
         <f>'UC3'!K13</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="33" t="str">
+      <c r="A18" s="29" t="str">
         <f>'UC3'!A14&amp;IF('UC3'!K14=TRUE," *","")&amp;IF('UC3'!I14="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0014</v>
       </c>
-      <c r="B18" s="34">
+      <c r="B18" s="24">
         <f>IF('UC3'!H14="","",'UC3'!H14)</f>
         <v>6</v>
       </c>
-      <c r="C18" s="35" t="str">
+      <c r="C18" t="str">
         <f>'UC3'!I14</f>
         <v>RISING</v>
       </c>
-      <c r="D18" s="34">
+      <c r="D18" s="24">
         <f>IF('UC3'!I14="RISING",'UC3'!H14,NA())</f>
         <v>6</v>
       </c>
-      <c r="E18" s="34" t="e">
+      <c r="E18" s="24" t="e">
         <f>IF('UC3'!I14="STABLE",'UC3'!H14,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F18" s="35">
+      <c r="F18">
         <f>'UC3'!C14</f>
         <v>2</v>
       </c>
-      <c r="G18" s="35" t="str">
+      <c r="G18" t="str">
         <f>IF('UC3'!J14="","",'UC3'!J14)</f>
         <v/>
       </c>
-      <c r="H18" s="36" t="b">
+      <c r="H18" s="30" t="b">
         <f>'UC3'!K14</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="33" t="str">
+      <c r="A19" s="29" t="str">
         <f>'UC3'!A15&amp;IF('UC3'!K15=TRUE," *","")&amp;IF('UC3'!I15="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0015</v>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="24">
         <f>IF('UC3'!H15="","",'UC3'!H15)</f>
         <v>-1</v>
       </c>
-      <c r="C19" s="35" t="str">
+      <c r="C19" t="str">
         <f>'UC3'!I15</f>
         <v>STABLE</v>
       </c>
-      <c r="D19" s="34" t="e">
+      <c r="D19" s="24" t="e">
         <f>IF('UC3'!I15="RISING",'UC3'!H15,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E19" s="34">
+      <c r="E19" s="24">
         <f>IF('UC3'!I15="STABLE",'UC3'!H15,NA())</f>
         <v>-1</v>
       </c>
-      <c r="F19" s="35">
+      <c r="F19">
         <f>'UC3'!C15</f>
         <v>2</v>
       </c>
-      <c r="G19" s="35" t="str">
+      <c r="G19" t="str">
         <f>IF('UC3'!J15="","",'UC3'!J15)</f>
         <v/>
       </c>
-      <c r="H19" s="36" t="b">
+      <c r="H19" s="30" t="b">
         <f>'UC3'!K15</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="33" t="str">
+      <c r="A20" s="29" t="str">
         <f>'UC3'!A16&amp;IF('UC3'!K16=TRUE," *","")&amp;IF('UC3'!I16="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0016 *</v>
       </c>
-      <c r="B20" s="34">
+      <c r="B20" s="24">
         <f>IF('UC3'!H16="","",'UC3'!H16)</f>
         <v>12</v>
       </c>
-      <c r="C20" s="35" t="str">
+      <c r="C20" t="str">
         <f>'UC3'!I16</f>
         <v>RISING</v>
       </c>
-      <c r="D20" s="34">
+      <c r="D20" s="24">
         <f>IF('UC3'!I16="RISING",'UC3'!H16,NA())</f>
         <v>12</v>
       </c>
-      <c r="E20" s="34" t="e">
+      <c r="E20" s="24" t="e">
         <f>IF('UC3'!I16="STABLE",'UC3'!H16,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="F20" s="35">
+      <c r="F20">
         <f>'UC3'!C16</f>
         <v>2</v>
       </c>
-      <c r="G20" s="35">
+      <c r="G20">
         <f>IF('UC3'!J16="","",'UC3'!J16)</f>
         <v>1</v>
       </c>
-      <c r="H20" s="36" t="b">
+      <c r="H20" s="30" t="b">
         <f>'UC3'!K16</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="37" t="str">
+      <c r="A21" s="31" t="str">
         <f>'UC3'!A17&amp;IF('UC3'!K17=TRUE," *","")&amp;IF('UC3'!I17="INSUFFICIENT_HISTORY"," (1 test)","")</f>
         <v>GL-0017 (1 test)</v>
       </c>
-      <c r="B21" s="38" t="str">
+      <c r="B21" s="32" t="str">
         <f>IF('UC3'!H17="","",'UC3'!H17)</f>
         <v/>
       </c>
@@ -7947,11 +7941,11 @@
         <f>'UC3'!I17</f>
         <v>INSUFFICIENT_HISTORY</v>
       </c>
-      <c r="D21" s="38" t="e">
+      <c r="D21" s="32" t="e">
         <f>IF('UC3'!I17="RISING",'UC3'!H17,NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="E21" s="38" t="e">
+      <c r="E21" s="32" t="e">
         <f>IF('UC3'!I17="STABLE",'UC3'!H17,NA())</f>
         <v>#N/A</v>
       </c>
@@ -7963,22 +7957,22 @@
         <f>IF('UC3'!J17="","",'UC3'!J17)</f>
         <v>0.91700000000000004</v>
       </c>
-      <c r="H21" s="39" t="b">
+      <c r="H21" s="33" t="b">
         <f>'UC3'!K17</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="46" t="s">
         <v>159</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -8003,75 +7997,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="40" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
+      <c r="A2" s="39" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="35"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="28" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="B6" s="36">
+      <c r="B6" s="30">
         <f>COUNTIF('UC4'!C:C,A6)</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="B7" s="39">
+      <c r="B7" s="33">
         <f>COUNTIF('UC4'!C:C,A7)</f>
         <v>1</v>
       </c>
@@ -8086,56 +8080,56 @@
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="31" t="s">
+      <c r="C24" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="D24" s="31" t="s">
+      <c r="D24" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="E24" s="43" t="s">
+      <c r="E24" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="43"/>
-      <c r="I24" s="43"/>
-      <c r="J24" s="44"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="42"/>
+      <c r="J24" s="43"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="33" t="str">
+      <c r="A25" s="29" t="str">
         <f>IF('UC4'!A2="","",'UC4'!A2)</f>
         <v>GL-0004</v>
       </c>
-      <c r="B25" s="35" t="str">
+      <c r="B25" t="str">
         <f>IF('UC4'!B2="","",'UC4'!B2)</f>
         <v>Olivia Brown</v>
       </c>
-      <c r="C25" s="35" t="str">
+      <c r="C25" t="str">
         <f>IF('UC4'!C2="","",'UC4'!C2)</f>
         <v>RESULT_NOT_RETURNED</v>
       </c>
-      <c r="D25" s="45">
+      <c r="D25" s="8">
         <f>IF('UC4'!E2="","",'UC4'!E2)</f>
-        <v>46087</v>
-      </c>
-      <c r="E25" s="46" t="str">
+        <v>46176</v>
+      </c>
+      <c r="E25" s="35" t="str">
         <f>IF('UC4'!D2="","",'UC4'!D2)</f>
         <v>Result OBS-0010 reported 2026-06-03 has no delivery record to a clinic</v>
       </c>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="47"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="35"/>
+      <c r="H25" s="35"/>
+      <c r="I25" s="35"/>
+      <c r="J25" s="36"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="37" t="str">
+      <c r="A26" s="31" t="str">
         <f>IF('UC4'!A3="","",'UC4'!A3)</f>
         <v>GL-0005</v>
       </c>
@@ -8147,19 +8141,19 @@
         <f>IF('UC4'!C3="","",'UC4'!C3)</f>
         <v>MULTI_PHARMACY_OVERLAP</v>
       </c>
-      <c r="D26" s="48">
+      <c r="D26" s="34">
         <f>IF('UC4'!E3="","",'UC4'!E3)</f>
         <v>46132</v>
       </c>
-      <c r="E26" s="49" t="str">
+      <c r="E26" s="37" t="str">
         <f>IF('UC4'!D3="","",'UC4'!D3)</f>
         <v>biguanide supplied by pharmacies 1 and 2 with overlapping supply from 2026-04-20</v>
       </c>
-      <c r="F26" s="49"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="49"/>
-      <c r="I26" s="49"/>
-      <c r="J26" s="50"/>
+      <c r="F26" s="37"/>
+      <c r="G26" s="37"/>
+      <c r="H26" s="37"/>
+      <c r="I26" s="37"/>
+      <c r="J26" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>